<commit_message>
virajes + recs cada 1s
he juntado la parte de alex y la mia
</commit_message>
<xml_diff>
--- a/RadarSeparation.xlsx
+++ b/RadarSeparation.xlsx
@@ -583,7 +583,7 @@
         <v>8.773637125929048</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q2" t="n">
         <v>3620.281073161436</v>
@@ -657,7 +657,7 @@
         <v>6.188205438717591</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q3" t="n">
         <v>2568.821135002041</v>
@@ -731,7 +731,7 @@
         <v>6.764160240530157</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q4" t="n">
         <v>5034.965146426352</v>
@@ -805,7 +805,7 @@
         <v>5.595231357403071</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q5" t="n">
         <v>3096.665451579348</v>
@@ -879,7 +879,7 @@
         <v>5.534080356031083</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q6" t="n">
         <v>2748.38285915433</v>
@@ -953,7 +953,7 @@
         <v>4.546314068276478</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q7" t="n">
         <v>2461.746954742964</v>
@@ -1027,7 +1027,7 @@
         <v>5.806694157981677</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q8" t="n">
         <v>2881.208240549883</v>
@@ -1101,7 +1101,7 @@
         <v>5.872458038059335</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q9" t="n">
         <v>4474.814509835956</v>
@@ -1175,7 +1175,7 @@
         <v>5.407894675713457</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q10" t="n">
         <v>2855.443111468849</v>
@@ -1249,7 +1249,7 @@
         <v>4.503266333807015</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q11" t="n">
         <v>2293.332029719426</v>
@@ -1315,7 +1315,7 @@
         <v>10.58936238927307</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q12" t="n">
         <v>7806.486706874188</v>
@@ -1389,7 +1389,7 @@
         <v>5.982933333820198</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q13" t="n">
         <v>3329.009676600119</v>
@@ -1463,7 +1463,7 @@
         <v>6.353294800544236</v>
       </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q14" t="n">
         <v>4420.051637189189</v>
@@ -1537,7 +1537,7 @@
         <v>4.948139942837459</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q15" t="n">
         <v>3069.895479392388</v>
@@ -1611,7 +1611,7 @@
         <v>5.322340678774827</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q16" t="n">
         <v>2600.011714745887</v>
@@ -1677,7 +1677,7 @@
         <v>5.621240373777285</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q17" t="n">
         <v>4843.310397846863</v>
@@ -1751,7 +1751,7 @@
         <v>4.850408902035884</v>
       </c>
       <c r="P18" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q18" t="n">
         <v>2561.280941328275</v>
@@ -1825,7 +1825,7 @@
         <v>5.875632483026255</v>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q19" t="n">
         <v>2888.514769119996</v>
@@ -1899,7 +1899,7 @@
         <v>7.638274582772553</v>
       </c>
       <c r="P20" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q20" t="n">
         <v>4369.218602597286</v>
@@ -1973,7 +1973,7 @@
         <v>4.643489412115283</v>
       </c>
       <c r="P21" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q21" t="n">
         <v>2476.22026030425</v>
@@ -2047,7 +2047,7 @@
         <v>6.485641188937064</v>
       </c>
       <c r="P22" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q22" t="n">
         <v>2667.128768143225</v>
@@ -2121,7 +2121,7 @@
         <v>7.549016481333314</v>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q23" t="n">
         <v>3823.152172915248</v>
@@ -2187,7 +2187,7 @@
         <v>18.99251701387163</v>
       </c>
       <c r="P24" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q24" t="n">
         <v>13054.48714363916</v>
@@ -2253,7 +2253,7 @@
         <v>14.83171854048441</v>
       </c>
       <c r="P25" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q25" t="n">
         <v>10950.7200594625</v>
@@ -2319,7 +2319,7 @@
         <v>8.60174057237732</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q26" t="n">
         <v>7816.700801354066</v>
@@ -2385,7 +2385,7 @@
         <v>19.35837255900584</v>
       </c>
       <c r="P27" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q27" t="n">
         <v>14975.70642134658</v>
@@ -2451,7 +2451,7 @@
         <v>10.56001636914746</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
@@ -2515,7 +2515,7 @@
         <v>17.21172945080025</v>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q29" t="n">
         <v>10267.85671534743</v>
@@ -2587,7 +2587,7 @@
         <v>5.367210993370685</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
@@ -2659,7 +2659,7 @@
         <v>5.622745361009136</v>
       </c>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q31" t="n">
         <v>2275.132486603803</v>
@@ -2733,7 +2733,7 @@
         <v>3.951043164932135</v>
       </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q32" t="n">
         <v>3590.607171739841</v>
@@ -2807,7 +2807,7 @@
         <v>4.112596652023546</v>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q33" t="n">
         <v>1420.052596834158</v>
@@ -2881,7 +2881,7 @@
         <v>3.780948906655723</v>
       </c>
       <c r="P34" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q34" t="n">
         <v>2116.458580716718</v>
@@ -2955,7 +2955,7 @@
         <v>3.650480445241904</v>
       </c>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q35" t="n">
         <v>1817.00352296109</v>
@@ -3029,7 +3029,7 @@
         <v>4.857614377691482</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q36" t="n">
         <v>3125.03285344732</v>
@@ -3103,7 +3103,7 @@
         <v>4.824619167676413</v>
       </c>
       <c r="P37" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q37" t="n">
         <v>3206.721852474182</v>
@@ -3177,7 +3177,7 @@
         <v>3.857990837093377</v>
       </c>
       <c r="P38" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q38" t="n">
         <v>1603.017139515698</v>
@@ -3251,7 +3251,7 @@
         <v>5.56812230228796</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q39" t="n">
         <v>2848.742137512773</v>
@@ -3325,7 +3325,7 @@
         <v>4.48962284566934</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q40" t="n">
         <v>1939.304262816515</v>
@@ -3399,7 +3399,7 @@
         <v>5.667871548392847</v>
       </c>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q41" t="n">
         <v>2656.813783798574</v>
@@ -3465,7 +3465,7 @@
         <v>5.805975023196801</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q42" t="n">
         <v>3721.762636722081</v>
@@ -3531,7 +3531,7 @@
         <v>4.124347824935252</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q43" t="n">
         <v>1998.517469002383</v>
@@ -3605,7 +3605,7 @@
         <v>3.991184292725319</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q44" t="n">
         <v>2095.17166970355</v>
@@ -3679,7 +3679,7 @@
         <v>3.860378978369986</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q45" t="n">
         <v>1866.651909683856</v>
@@ -3753,7 +3753,7 @@
         <v>5.786357054594571</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q46" t="n">
         <v>3579.254950614478</v>
@@ -3827,7 +3827,7 @@
         <v>5.533705813538385</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q47" t="n">
         <v>2885.875056065668</v>
@@ -3901,7 +3901,7 @@
         <v>4.455252538810387</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q48" t="n">
         <v>1337.453392198467</v>
@@ -3975,7 +3975,7 @@
         <v>5.872083012711612</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q49" t="n">
         <v>3821.732870999234</v>
@@ -4049,7 +4049,7 @@
         <v>3.623140689178709</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q50" t="n">
         <v>1636.397751006394</v>
@@ -4123,7 +4123,7 @@
         <v>3.976563956729924</v>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q51" t="n">
         <v>1866.415261095229</v>
@@ -4197,7 +4197,7 @@
         <v>3.911731439487217</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q52" t="n">
         <v>2698.56229100568</v>
@@ -4271,7 +4271,7 @@
         <v>4.017921902036949</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q53" t="n">
         <v>1805.847311815819</v>
@@ -4345,7 +4345,7 @@
         <v>5.492453731270511</v>
       </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q54" t="n">
         <v>2597.189049509203</v>
@@ -4419,7 +4419,7 @@
         <v>4.081867939013645</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q55" t="n">
         <v>2164.372375258797</v>
@@ -4493,7 +4493,7 @@
         <v>6.26584955175126</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q56" t="n">
         <v>3479.497174798933</v>
@@ -4567,7 +4567,7 @@
         <v>3.241426660720493</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q57" t="n">
         <v>1715.162683711208</v>
@@ -4639,7 +4639,7 @@
         <v>4.905766007393035</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr">
@@ -4711,7 +4711,7 @@
         <v>4.390820103969347</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q59" t="n">
         <v>2345.022471251741</v>
@@ -4785,7 +4785,7 @@
         <v>3.745346442226908</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr">
@@ -4857,7 +4857,7 @@
         <v>5.11578298245241</v>
       </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q61" t="n">
         <v>3276.196329794571</v>
@@ -4931,7 +4931,7 @@
         <v>4.548553283365578</v>
       </c>
       <c r="P62" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="inlineStr">
@@ -5003,7 +5003,7 @@
         <v>3.324498844707619</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q63" t="n">
         <v>1925.070657404491</v>
@@ -5077,7 +5077,7 @@
         <v>4.246056090554172</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q64" t="n">
         <v>3070.214301018874</v>
@@ -5151,7 +5151,7 @@
         <v>4.56045972170778</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q65" t="n">
         <v>2162.705467055987</v>
@@ -5225,7 +5225,7 @@
         <v>4.196303521158117</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q66" t="n">
         <v>1978.119549624547</v>
@@ -5299,7 +5299,7 @@
         <v>3.827904010745061</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q67" t="n">
         <v>2319.914589190835</v>
@@ -5373,7 +5373,7 @@
         <v>4.77448126077643</v>
       </c>
       <c r="P68" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q68" t="n">
         <v>2439.160070368576</v>
@@ -5447,7 +5447,7 @@
         <v>4.753478985811091</v>
       </c>
       <c r="P69" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q69" t="n">
         <v>3017.588237808717</v>
@@ -5521,7 +5521,7 @@
         <v>6.125219515616166</v>
       </c>
       <c r="P70" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q70" t="n">
         <v>3861.290128105628</v>
@@ -5595,7 +5595,7 @@
         <v>6.070820738236529</v>
       </c>
       <c r="P71" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q71" t="n">
         <v>4575.011507975029</v>
@@ -5669,7 +5669,7 @@
         <v>3.877299993693755</v>
       </c>
       <c r="P72" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q72" t="n">
         <v>2663.761158410617</v>
@@ -5743,7 +5743,7 @@
         <v>4.652684370068189</v>
       </c>
       <c r="P73" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q73" t="n">
         <v>2031.869646984498</v>
@@ -5817,7 +5817,7 @@
         <v>3.544200715742492</v>
       </c>
       <c r="P74" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q74" t="n">
         <v>1835.824019466443</v>
@@ -5891,7 +5891,7 @@
         <v>4.505848836325718</v>
       </c>
       <c r="P75" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q75" t="n">
         <v>1873.124539617948</v>
@@ -5957,7 +5957,7 @@
         <v>11.54048720384428</v>
       </c>
       <c r="P76" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q76" t="n">
         <v>7993.022027145769</v>
@@ -6031,7 +6031,7 @@
         <v>5.091992253319329</v>
       </c>
       <c r="P77" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q77" t="n">
         <v>3537.477605795105</v>
@@ -6105,7 +6105,7 @@
         <v>4.770289090981912</v>
       </c>
       <c r="P78" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q78" t="n">
         <v>2302.559300333876</v>
@@ -6179,7 +6179,7 @@
         <v>8.130794134857354</v>
       </c>
       <c r="P79" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q79" t="n">
         <v>4653.48823325286</v>
@@ -6253,7 +6253,7 @@
         <v>6.531934832615485</v>
       </c>
       <c r="P80" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q80" t="n">
         <v>2437.851859320508</v>
@@ -6327,7 +6327,7 @@
         <v>4.756816180152658</v>
       </c>
       <c r="P81" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q81" t="n">
         <v>2792.781275024198</v>
@@ -6401,7 +6401,7 @@
         <v>6.243419129208053</v>
       </c>
       <c r="P82" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q82" t="n">
         <v>2890.568018253165</v>
@@ -6475,7 +6475,7 @@
         <v>6.217966200635963</v>
       </c>
       <c r="P83" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q83" t="n">
         <v>4522.451610627212</v>
@@ -6549,7 +6549,7 @@
         <v>4.261480341091596</v>
       </c>
       <c r="P84" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q84" t="n">
         <v>1473.521451456588</v>
@@ -6615,7 +6615,7 @@
         <v>37.41076996100543</v>
       </c>
       <c r="P85" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q85" t="n">
         <v>29029.5686546914</v>
@@ -6681,7 +6681,7 @@
         <v>6.88097280634908</v>
       </c>
       <c r="P86" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q86" t="n">
         <v>5112.348556225783</v>
@@ -6747,7 +6747,7 @@
         <v>9.532071976676812</v>
       </c>
       <c r="P87" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q87" t="n">
         <v>5745.408523189255</v>
@@ -6821,7 +6821,7 @@
         <v>6.946164193986857</v>
       </c>
       <c r="P88" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q88" t="n">
         <v>4039.010865980704</v>
@@ -6895,7 +6895,7 @@
         <v>6.517339405767062</v>
       </c>
       <c r="P89" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q89" t="n">
         <v>3228.993168913027</v>
@@ -6969,7 +6969,7 @@
         <v>3.816568987320708</v>
       </c>
       <c r="P90" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q90" t="n">
         <v>1978.363041750179</v>
@@ -7043,7 +7043,7 @@
         <v>5.093441544317968</v>
       </c>
       <c r="P91" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q91" t="n">
         <v>2839.374080892851</v>
@@ -7117,7 +7117,7 @@
         <v>5.470129057825526</v>
       </c>
       <c r="P92" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q92" t="n">
         <v>3078.309411513685</v>
@@ -7183,7 +7183,7 @@
         <v>27.70303273102304</v>
       </c>
       <c r="P93" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q93" t="n">
         <v>18724.42392011629</v>
@@ -7257,7 +7257,7 @@
         <v>5.474829877423945</v>
       </c>
       <c r="P94" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q94" t="n">
         <v>2369.187867016654</v>
@@ -7331,7 +7331,7 @@
         <v>5.7430678787302</v>
       </c>
       <c r="P95" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q95" t="n">
         <v>2849.406613925066</v>
@@ -7397,7 +7397,7 @@
         <v>15.38607608225034</v>
       </c>
       <c r="P96" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q96" t="n">
         <v>12833.15444210844</v>
@@ -7471,7 +7471,7 @@
         <v>5.758127947888689</v>
       </c>
       <c r="P97" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q97" t="n">
         <v>2981.150509081503</v>
@@ -7545,7 +7545,7 @@
         <v>3.918232073722256</v>
       </c>
       <c r="P98" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q98" t="n">
         <v>1674.073422191074</v>
@@ -7619,7 +7619,7 @@
         <v>5.81874615140462</v>
       </c>
       <c r="P99" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q99" t="n">
         <v>3445.981281148013</v>
@@ -7693,7 +7693,7 @@
         <v>3.832435817535283</v>
       </c>
       <c r="P100" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q100" t="n">
         <v>2175.736563990438</v>
@@ -7759,7 +7759,7 @@
         <v>18.59659885672986</v>
       </c>
       <c r="P101" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q101" t="n">
         <v>66895.94417845955</v>
@@ -7833,7 +7833,7 @@
         <v>5.026937648058869</v>
       </c>
       <c r="P102" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q102" t="n">
         <v>3269.741090812225</v>
@@ -7907,7 +7907,7 @@
         <v>8.04989772365426</v>
       </c>
       <c r="P103" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q103" t="n">
         <v>2752.43385046948</v>
@@ -7973,7 +7973,7 @@
         <v>6.167178506328621</v>
       </c>
       <c r="P104" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q104" t="n">
         <v>5812.772450726096</v>
@@ -8047,7 +8047,7 @@
         <v>4.283569991853439</v>
       </c>
       <c r="P105" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q105" t="n">
         <v>2183.855455171256</v>
@@ -8113,7 +8113,7 @@
         <v>5.458747931967979</v>
       </c>
       <c r="P106" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q106" t="n">
         <v>2867.263394085484</v>
@@ -8179,7 +8179,7 @@
         <v>5.050037051585375</v>
       </c>
       <c r="P107" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q107" t="n">
         <v>2929.262171011406</v>
@@ -8253,7 +8253,7 @@
         <v>6.368879213056079</v>
       </c>
       <c r="P108" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q108" t="n">
         <v>3909.901724406096</v>
@@ -8319,7 +8319,7 @@
         <v>12.92683526310222</v>
       </c>
       <c r="P109" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q109" t="n">
         <v>8321.694843742804</v>
@@ -8393,7 +8393,7 @@
         <v>5.632456073133972</v>
       </c>
       <c r="P110" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q110" t="n">
         <v>3096.078285076505</v>
@@ -8467,7 +8467,7 @@
         <v>5.482307342910589</v>
       </c>
       <c r="P111" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q111" t="n">
         <v>3466.901402590073</v>
@@ -8541,7 +8541,7 @@
         <v>4.163074437719279</v>
       </c>
       <c r="P112" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q112" t="n">
         <v>2405.683541346745</v>
@@ -8615,7 +8615,7 @@
         <v>7.625488947801215</v>
       </c>
       <c r="P113" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q113" t="n">
         <v>3829.450633867101</v>
@@ -8689,7 +8689,7 @@
         <v>6.116691645125452</v>
       </c>
       <c r="P114" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q114" t="n">
         <v>4182.457946118417</v>
@@ -8755,7 +8755,7 @@
         <v>12.71299663477823</v>
       </c>
       <c r="P115" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q115" t="n">
         <v>6941.01811196804</v>
@@ -8829,7 +8829,7 @@
         <v>4.252799092364027</v>
       </c>
       <c r="P116" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q116" t="n">
         <v>1662.390470744966</v>
@@ -8903,7 +8903,7 @@
         <v>6.172882528447686</v>
       </c>
       <c r="P117" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q117" t="n">
         <v>3702.90811295111</v>
@@ -8977,7 +8977,7 @@
         <v>4.25534751062803</v>
       </c>
       <c r="P118" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q118" t="n">
         <v>2366.369238485157</v>
@@ -9043,7 +9043,7 @@
         <v>17.88979168922451</v>
       </c>
       <c r="P119" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q119" t="n">
         <v>10913.28158221424</v>

</xml_diff>